<commit_message>
Release Version 2: Updated background, revised experience details, added Version 1 link, and uploaded latest resume.
</commit_message>
<xml_diff>
--- a/wwwroot/Strorage/SystemRegistrations.xlsx
+++ b/wwwroot/Strorage/SystemRegistrations.xlsx
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" fullPrecision="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>SystemId</t>
   </si>
@@ -43,13 +43,29 @@
   </si>
   <si>
     <t>RegisteredAt</t>
+  </si>
+  <si>
+    <t>Win32_Mozilla/5.0 (Windows NT 10.0; Win64; x64) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/145.0.0.0 Safari/537.36</t>
+  </si>
+  <si>
+    <t>OS: Win32, Browser: Mozilla/5.0 (Windows NT 10.0; Win64; x64) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/145.0.0.0 Safari/537.36</t>
+  </si>
+  <si>
+    <t>22-03-26 10:53:44 AM</t>
+  </si>
+  <si>
+    <t>22-03-26 12:38:30 PM</t>
+  </si>
+  <si>
+    <t>22-03-26 12:41:38 PM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -394,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83229955-CCFF-474F-9A58-7F0542038532}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -402,18 +418,52 @@
     <col min="3" max="3" width="42.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="0" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>